<commit_message>
Aktueller Stand nach Timo
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\korbinian.zacherl\Documents\UiPath\XÖV\XÖV\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\timotheus.vrettos\develop\develop_RPA\uipath-rpa_XOV\XÖV\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0E6C47B-C4F7-4B13-A1A3-2C1955A6F5D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10A96881-B2F2-4461-8867-692BDE9FB85D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="73">
   <si>
     <t>Name</t>
   </si>
@@ -241,13 +241,16 @@
   </si>
   <si>
     <t>rpa009_Webex_RoomID</t>
+  </si>
+  <si>
+    <t>rpa021_Excluded_Workers</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -277,6 +280,12 @@
       <color theme="10"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF464E55"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -299,7 +308,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -310,6 +319,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -626,12 +638,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z998"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="43.5703125" customWidth="1"/>
+    <col min="1" max="1" width="43.5546875" customWidth="1"/>
     <col min="2" max="2" width="43" customWidth="1"/>
-    <col min="3" max="3" width="81.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="3" max="3" width="81.44140625" customWidth="1"/>
+    <col min="4" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -677,7 +689,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="45">
+    <row r="3" spans="1:26" ht="43.2">
       <c r="A3" s="2" t="s">
         <v>31</v>
       </c>
@@ -687,7 +699,7 @@
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="30">
+    <row r="5" spans="1:26" ht="28.8">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -1722,12 +1734,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z998"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" customWidth="1"/>
-    <col min="3" max="3" width="75.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="3" max="3" width="75.44140625" customWidth="1"/>
+    <col min="4" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -1764,7 +1776,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="30">
+    <row r="2" spans="1:26" ht="28.8">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1775,7 +1787,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="30">
+    <row r="3" spans="1:26" ht="28.8">
       <c r="A3" t="s">
         <v>44</v>
       </c>
@@ -1786,7 +1798,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="45">
+    <row r="4" spans="1:26" ht="43.2">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -1797,7 +1809,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:26">
+    <row r="5" spans="1:26" ht="14.4">
       <c r="A5" t="s">
         <v>46</v>
       </c>
@@ -1828,7 +1840,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:26">
+    <row r="9" spans="1:26" ht="14.4">
       <c r="A9" t="s">
         <v>48</v>
       </c>
@@ -1839,8 +1851,8 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:26"/>
-    <row r="11" spans="1:26">
+    <row r="10" spans="1:26" ht="14.4"/>
+    <row r="11" spans="1:26" ht="14.4">
       <c r="A11" t="s">
         <v>49</v>
       </c>
@@ -1851,7 +1863,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="12" spans="1:26">
+    <row r="12" spans="1:26" ht="14.4">
       <c r="A12" t="s">
         <v>50</v>
       </c>
@@ -1862,7 +1874,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="13" spans="1:26">
+    <row r="13" spans="1:26" ht="14.4">
       <c r="A13" t="s">
         <v>51</v>
       </c>
@@ -1873,7 +1885,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="14" spans="1:26">
+    <row r="14" spans="1:26" ht="14.4">
       <c r="A14" t="s">
         <v>53</v>
       </c>
@@ -1884,7 +1896,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="15" spans="1:26">
+    <row r="15" spans="1:26" ht="14.4">
       <c r="A15" t="s">
         <v>55</v>
       </c>
@@ -1986,7 +1998,7 @@
       </c>
     </row>
     <row r="26" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="27" spans="1:3" ht="45">
+    <row r="27" spans="1:3" ht="28.8">
       <c r="A27" t="s">
         <v>40</v>
       </c>
@@ -2976,12 +2988,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.85546875" customWidth="1"/>
-    <col min="2" max="2" width="30.140625" customWidth="1"/>
-    <col min="3" max="3" width="60.28515625" customWidth="1"/>
-    <col min="4" max="26" width="65.42578125" customWidth="1"/>
+    <col min="1" max="1" width="31.88671875" customWidth="1"/>
+    <col min="2" max="2" width="30.109375" customWidth="1"/>
+    <col min="3" max="3" width="60.33203125" customWidth="1"/>
+    <col min="4" max="26" width="65.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -3020,7 +3032,14 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="2" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A2" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="5" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>